<commit_message>
chore: atualiza relatório macro (2026-08)
</commit_message>
<xml_diff>
--- a/projetos/relatorio-macro-excel/relatorio_macro.xlsx
+++ b/projetos/relatorio-macro-excel/relatorio_macro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selic" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Câmbio" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IPCA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Selic" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Câmbio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="IPCA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -221,14 +221,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -251,7 +251,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="E85D04"/>
               </a:solidFill>
@@ -261,19 +261,19 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Selic'!$A$5:$A$190</f>
+              <f>'Selic'!$A$5:$A$191</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Selic'!$B$5:$B$190</f>
+              <f>'Selic'!$B$5:$B$191</f>
             </numRef>
           </val>
         </ser>
@@ -309,14 +309,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -339,7 +339,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="E85D04"/>
               </a:solidFill>
@@ -349,7 +349,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -397,14 +397,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -427,7 +427,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="E85D04"/>
               </a:solidFill>
@@ -437,7 +437,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -485,7 +485,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -500,9 +500,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -512,7 +512,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -527,9 +527,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -539,7 +539,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -554,9 +554,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -894,7 +894,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Gerado automaticamente em 16/07/2026 19:08 · Fonte: Banco Central do Brasil (API SGS)</t>
+          <t>Gerado automaticamente em 01/08/2026 13:41 · Fonte: Banco Central do Brasil (API SGS)</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
     <row r="8">
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>14,40% a.a.</t>
+          <t>14,15% a.a.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -945,7 +945,7 @@
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>em 2026-06</t>
+          <t>em 2026-07</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B190"/>
+  <dimension ref="A1:B191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2873,7 +2873,17 @@
         </is>
       </c>
       <c r="B190" s="14" t="n">
-        <v>14.4</v>
+        <v>14.29</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="11" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B191" s="12" t="n">
+        <v>14.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>